<commit_message>
Development is in progress
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP22_RequisitosCalidadPedidoProveedor\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5F87597-2912-4FC7-BE79-519B7D459F47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{795639C8-8DBF-43C1-BB4E-CB5F533258F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="95">
   <si>
     <t>Name</t>
   </si>
@@ -235,33 +235,6 @@
     <t>Nombres de disposicion en SAP</t>
   </si>
   <si>
-    <t>ODM_TimeoutShort</t>
-  </si>
-  <si>
-    <t>ODM_TimeoutMedium</t>
-  </si>
-  <si>
-    <t>ODM_TimeoutLong</t>
-  </si>
-  <si>
-    <t>Timeout corto para interactuar en ODM</t>
-  </si>
-  <si>
-    <t>Timeout medio para interactuar en ODM</t>
-  </si>
-  <si>
-    <t>Timeout largo para interactuar en ODM</t>
-  </si>
-  <si>
-    <t>ODM_URL</t>
-  </si>
-  <si>
-    <t>La URL para abrir la app de ODM</t>
-  </si>
-  <si>
-    <t>ODM_Creds</t>
-  </si>
-  <si>
     <t>ISR_InitialInpuPath</t>
   </si>
   <si>
@@ -274,15 +247,6 @@
     <t>SEGUIMIENTO REPUESTOS {0}.xlsm</t>
   </si>
   <si>
-    <t>ISR_SAPBatchIntervals</t>
-  </si>
-  <si>
-    <t>SAPBatchIntervals</t>
-  </si>
-  <si>
-    <t>Intervalos de lotes para ingresarlos a las transacciones SAP, el guion separa el intervalo y el punto y coma separa el par</t>
-  </si>
-  <si>
     <t>ISR_MacroName</t>
   </si>
   <si>
@@ -292,18 +256,6 @@
     <t>Nombre de la macro a ejecutar dentro del reporte Seguimiento Respuestos</t>
   </si>
   <si>
-    <t>Datos de Validación Compras</t>
-  </si>
-  <si>
-    <t>Credenciales para logueo en ODM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nombre de la hoja del reporte ODM </t>
-  </si>
-  <si>
-    <t>ODM_SheetName</t>
-  </si>
-  <si>
     <t>Data</t>
   </si>
   <si>
@@ -313,64 +265,12 @@
     <t>Nombre de la hoja del reportes SAP</t>
   </si>
   <si>
-    <t>AMP06_00_InformeSeguimientoRepuestos</t>
-  </si>
-  <si>
-    <t>saplogon.exe;EXCEL;msedge.exe</t>
-  </si>
-  <si>
-    <t>ISR_FinalFolderReportPath</t>
-  </si>
-  <si>
     <t>Ruta de la carpeta para guardar el reporte final</t>
   </si>
   <si>
     <t>FinalFolderReportPath</t>
   </si>
   <si>
-    <t>Intervalo de lotes transacción</t>
-  </si>
-  <si>
-    <t>BatchTransactionZSD053</t>
-  </si>
-  <si>
-    <t>35000000;35999999</t>
-  </si>
-  <si>
-    <t>ODM_MenuName</t>
-  </si>
-  <si>
-    <t>Nombre del menú en ODM</t>
-  </si>
-  <si>
-    <t>RangeData</t>
-  </si>
-  <si>
-    <t>Transaction;Range
-ZMG002_01;B2
-ZMM026;C2
-LX02;E2
-COHV;C2
-ZCO017;B2
-ZPP029_1;A2
-MB52;C2
-ZSD053;C2
-LT23;C2
-VL06O;A2</t>
-  </si>
-  <si>
-    <t>DefaultRange</t>
-  </si>
-  <si>
-    <t>B2</t>
-  </si>
-  <si>
-    <t>Los rangos para cada una de las transacciones</t>
-  </si>
-  <si>
-    <t>El rango por defecto</t>
-  </si>
-  <si>
     <t>LayOutSAP</t>
   </si>
   <si>
@@ -383,55 +283,57 @@
     <t>C:\Users\aci-cns\Documents\Test UiPath\Informe seguimiento Repuestos\Exceptions_Screenshots</t>
   </si>
   <si>
-    <t>SplitBatchIntervalZMM026</t>
-  </si>
-  <si>
-    <t>Valor inicial para partir los intervalos de los lotes a la transacción</t>
-  </si>
-  <si>
-    <t>SplitBatchIntervalCOHV</t>
-  </si>
-  <si>
-    <t>SplitBatchIntervalZPP029_1</t>
+    <t>AMP22_RequisitosCalidadPedidoProveedor</t>
+  </si>
+  <si>
+    <t>saplogon.exe;EXCEL;chrome.exe</t>
+  </si>
+  <si>
+    <t>Credenciales para logueo en Share Point</t>
+  </si>
+  <si>
+    <t>SharePoint_Creds</t>
+  </si>
+  <si>
+    <t>RCPP_FinalFolderReportPath</t>
+  </si>
+  <si>
+    <t>SP_TimeoutMedium</t>
+  </si>
+  <si>
+    <t>Timeout medio para interactuar en Share Point</t>
+  </si>
+  <si>
+    <t>SP_TimeoutShort</t>
+  </si>
+  <si>
+    <t>Timeout corto para interactuar en Share Point</t>
+  </si>
+  <si>
+    <t>SP_TimeoutLong</t>
+  </si>
+  <si>
+    <t>Timeout largo  para interactuar en Share Point</t>
+  </si>
+  <si>
+    <t>ZMM026</t>
+  </si>
+  <si>
+    <t>Primera transacción a ejecutar en SAP</t>
+  </si>
+  <si>
+    <t>FirstTransaction</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -540,12 +442,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -560,32 +468,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -802,7 +703,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z1000"/>
+  <dimension ref="A1:Z993"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -872,7 +773,7 @@
         <v>9</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>10</v>
@@ -883,7 +784,7 @@
         <v>53</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>54</v>
@@ -901,141 +802,81 @@
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>85</v>
+      <c r="A7" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>77</v>
+      <c r="A8" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>68</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>84</v>
+      <c r="A9" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>72</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>88</v>
+      <c r="A10" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>78</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
-        <v>97</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>98</v>
+      <c r="A11" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>92</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="19" t="s">
-        <v>111</v>
-      </c>
-      <c r="B12" s="20">
-        <v>35002000</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="B13" s="20">
-        <v>35002000</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="21" t="s">
-        <v>114</v>
-      </c>
-      <c r="B14" s="20">
-        <v>35002000</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="15" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="B15" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
-        <v>103</v>
-      </c>
-      <c r="B16" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="18" t="s">
-        <v>107</v>
-      </c>
-      <c r="B17" s="18" t="s">
-        <v>108</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="34" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="35" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1217,13 +1058,13 @@
     <row r="211" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="212" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="213" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="214" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="215" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="216" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="217" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="218" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="219" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="220" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="214" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="215" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="216" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="217" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="218" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="219" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="220" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="221" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="222" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="223" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1997,15 +1838,8 @@
     <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <phoneticPr fontId="20" type="noConversion"/>
+  <phoneticPr fontId="16" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -2083,7 +1917,7 @@
         <v>17</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>110</v>
+        <v>80</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
@@ -3181,7 +3015,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Z985"/>
+  <dimension ref="A1:Z982"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="4" customWidth="1"/>
@@ -3192,251 +3026,212 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
-      <c r="N1" s="11"/>
-      <c r="O1" s="11"/>
-      <c r="P1" s="11"/>
-      <c r="Q1" s="11"/>
-      <c r="R1" s="11"/>
-      <c r="S1" s="11"/>
-      <c r="T1" s="11"/>
-      <c r="U1" s="11"/>
-      <c r="V1" s="11"/>
-      <c r="W1" s="11"/>
-      <c r="X1" s="11"/>
-      <c r="Y1" s="11"/>
-      <c r="Z1" s="11"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
+      <c r="R1" s="10"/>
+      <c r="S1" s="10"/>
+      <c r="T1" s="10"/>
+      <c r="U1" s="10"/>
+      <c r="V1" s="10"/>
+      <c r="W1" s="10"/>
+      <c r="X1" s="10"/>
+      <c r="Y1" s="10"/>
+      <c r="Z1" s="10"/>
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="9" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="9" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="9" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="C6" s="10" t="s">
+      <c r="A6" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="10" t="s">
-        <v>68</v>
+      <c r="D6" s="9" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="C7" s="10" t="s">
+      <c r="A7" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="10" t="s">
-        <v>69</v>
+      <c r="D7" s="9" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="C8" s="10" t="s">
+      <c r="A8" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>70</v>
+      <c r="D8" s="9" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B9" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="C9" s="10" t="s">
+      <c r="B9" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="9" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="C10" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="13" t="s">
-        <v>94</v>
+      <c r="D10" s="11" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="9" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="9" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="B13" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>72</v>
-      </c>
     </row>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" s="12" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="15" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" s="15" t="s">
-        <v>100</v>
-      </c>
-    </row>
+    <row r="14" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3623,9 +3418,9 @@
     <row r="200" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="201" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="202" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="203" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="204" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="205" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="203" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="204" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="205" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="206" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="207" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="208" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -4403,9 +4198,6 @@
     <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape" r:id="rId1"/>

</xml_diff>